<commit_message>
Update workload report and add new account detail files
- Updated the existing workload report for March 2026.
- Added new Excel files for account details: gl_1775102264925 and gl_1775102272564.
</commit_message>
<xml_diff>
--- a/tmp_reports/workload-2026-03.xlsx
+++ b/tmp_reports/workload-2026-03.xlsx
@@ -56,6 +56,9 @@
     <t>% ARA</t>
   </si>
   <si>
+    <t>% C2L</t>
+  </si>
+  <si>
     <t>% SHIR</t>
   </si>
   <si>
@@ -66,9 +69,6 @@
   </si>
   <si>
     <t>% CH</t>
-  </si>
-  <si>
-    <t>% C2L</t>
   </si>
   <si>
     <t>% CEL</t>
@@ -899,10 +899,10 @@
         <v>0</v>
       </c>
       <c r="P3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="6">
         <v>51.19</v>
-      </c>
-      <c r="Q3" s="6">
-        <v>0</v>
       </c>
       <c r="R3" s="6">
         <v>0</v>
@@ -1088,10 +1088,10 @@
         <v>0</v>
       </c>
       <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
         <v>79.83</v>
-      </c>
-      <c r="O6" s="6">
-        <v>0</v>
       </c>
       <c r="P6" s="6">
         <v>0</v>
@@ -1123,13 +1123,13 @@
         <v>176</v>
       </c>
       <c r="D7" s="7">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="E7" s="7">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="F7" s="7">
-        <v>13.07</v>
+        <v>3.98</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>29</v>
@@ -1138,7 +1138,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="7">
-        <v>86.93</v>
+        <v>96.02</v>
       </c>
       <c r="J7" s="7">
         <v>0</v>
@@ -1738,19 +1738,19 @@
         <v>0</v>
       </c>
       <c r="N16" s="7">
-        <v>0</v>
+        <v>32.42</v>
       </c>
       <c r="O16" s="7">
+        <v>0</v>
+      </c>
+      <c r="P16" s="7">
         <v>64.8</v>
       </c>
-      <c r="P16" s="7">
-        <v>0</v>
-      </c>
       <c r="Q16" s="7">
         <v>0</v>
       </c>
       <c r="R16" s="7">
-        <v>32.42</v>
+        <v>0</v>
       </c>
       <c r="S16" s="7">
         <v>11.36</v>
@@ -1936,10 +1936,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="6">
+        <v>0</v>
+      </c>
+      <c r="P19" s="6">
         <v>9.09</v>
-      </c>
-      <c r="P19" s="6">
-        <v>0</v>
       </c>
       <c r="Q19" s="6">
         <v>0</v>
@@ -1998,10 +1998,10 @@
         <v>0</v>
       </c>
       <c r="N20" s="6">
+        <v>0</v>
+      </c>
+      <c r="O20" s="6">
         <v>3.5</v>
-      </c>
-      <c r="O20" s="6">
-        <v>0</v>
       </c>
       <c r="P20" s="6">
         <v>0</v>
@@ -2072,10 +2072,10 @@
         <v>0</v>
       </c>
       <c r="Q21" s="6">
+        <v>0</v>
+      </c>
+      <c r="R21" s="6">
         <v>50.28</v>
-      </c>
-      <c r="R21" s="6">
-        <v>0</v>
       </c>
       <c r="S21" s="6">
         <v>0</v>
@@ -2293,13 +2293,13 @@
         <v>176</v>
       </c>
       <c r="D25" s="7">
-        <v>152.03</v>
+        <v>211.45</v>
       </c>
       <c r="E25" s="7">
-        <v>23.97</v>
+        <v>0</v>
       </c>
       <c r="F25" s="7">
-        <v>13.62</v>
+        <v>0</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>29</v>
@@ -2323,7 +2323,7 @@
         <v>23.17</v>
       </c>
       <c r="N25" s="7">
-        <v>0</v>
+        <v>51.52</v>
       </c>
       <c r="O25" s="7">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="7">
-        <v>17.76</v>
+        <v>0</v>
       </c>
       <c r="S25" s="7">
         <v>0</v>
@@ -2628,10 +2628,10 @@
         <v>91</v>
       </c>
       <c r="E10">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="F10">
-        <v>86.93</v>
+        <v>96.02</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -3122,16 +3122,16 @@
         <v>69</v>
       </c>
       <c r="C35" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="D35" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E35">
-        <v>80</v>
+        <v>90.67</v>
       </c>
       <c r="F35">
-        <v>45.45</v>
+        <v>51.52</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -3142,16 +3142,16 @@
         <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D36" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E36">
-        <v>40.78</v>
+        <v>80</v>
       </c>
       <c r="F36">
-        <v>23.17</v>
+        <v>45.45</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -3162,16 +3162,16 @@
         <v>69</v>
       </c>
       <c r="C37" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="D37" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="E37">
-        <v>31.25</v>
+        <v>40.78</v>
       </c>
       <c r="F37">
-        <v>17.76</v>
+        <v>23.17</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>